<commit_message>
V2 of the MK1 Design
</commit_message>
<xml_diff>
--- a/_MK-1_/NeoSumec_MK-1_MECH.xlsx
+++ b/_MK-1_/NeoSumec_MK-1_MECH.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vadim\GitHub\NeoSumec\NeoSumec-MiniSumo-MECH\_MK-1_\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FAB970-D325-41C5-8077-1D03F7F348C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D98AE73-7970-4FAB-8A3B-9AA7BA3AF067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E70E74EA-06C0-433E-BC4D-5A3409939100}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
   <si>
     <t>Name</t>
   </si>
@@ -53,9 +53,6 @@
     <t>M3x20 Torx</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>M3x16 Torx</t>
   </si>
   <si>
@@ -104,14 +101,44 @@
     <t>M3x8 Torx</t>
   </si>
   <si>
-    <t>Spoj těl</t>
+    <t>Norm</t>
+  </si>
+  <si>
+    <t>DIN 934</t>
+  </si>
+  <si>
+    <t>DIN 916</t>
+  </si>
+  <si>
+    <t>ISO 14581</t>
+  </si>
+  <si>
+    <t>ISO 14583</t>
+  </si>
+  <si>
+    <t>ISO 14580</t>
+  </si>
+  <si>
+    <t>Vrchni spoj tel, PCB, Vrch</t>
+  </si>
+  <si>
+    <t>Spodni spoj těl</t>
+  </si>
+  <si>
+    <t>SenRigFront</t>
+  </si>
+  <si>
+    <t>M3x4 Torx</t>
+  </si>
+  <si>
+    <t>DIN 562</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +162,13 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -526,17 +560,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C58A2579-B6B4-43B1-AA5E-44312C298E05}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="4.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.109375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="10.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="4.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.21875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15" style="1" customWidth="1"/>
-    <col min="5" max="16384" width="4.44140625" style="1"/>
+    <col min="4" max="4" width="21.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="4.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -547,40 +582,49 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="E2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1">
         <v>4</v>
@@ -589,104 +633,159 @@
         <v>2</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="1">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="1">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D7" s="1" t="s">
+      <c r="B9" s="1">
+        <v>2</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1">
+        <v>4</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="E10" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="E11" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="1">
-        <v>1</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>16</v>
-      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{517062B2-C385-4292-8D30-9A915CC87D3F}"/>
-    <hyperlink ref="C8" r:id="rId2" xr:uid="{DF4E92D8-3D63-4001-A402-5388A1064A13}"/>
-    <hyperlink ref="C7" r:id="rId3" xr:uid="{CD317AC6-70D6-4FAA-82DC-062D351DD800}"/>
+    <hyperlink ref="C10" r:id="rId2" xr:uid="{DF4E92D8-3D63-4001-A402-5388A1064A13}"/>
+    <hyperlink ref="C9" r:id="rId3" xr:uid="{CD317AC6-70D6-4FAA-82DC-062D351DD800}"/>
     <hyperlink ref="C3" r:id="rId4" xr:uid="{9C5AFEAA-C950-4E19-8D53-8DAA31C707E1}"/>
-    <hyperlink ref="C9" r:id="rId5" xr:uid="{7454B801-582F-42C8-9E89-E8EDF2B0335C}"/>
-    <hyperlink ref="C10" r:id="rId6" xr:uid="{F47098D1-FCD7-4195-A6D3-516CD065EAF2}"/>
+    <hyperlink ref="C11" r:id="rId5" xr:uid="{7454B801-582F-42C8-9E89-E8EDF2B0335C}"/>
+    <hyperlink ref="C12" r:id="rId6" xr:uid="{F47098D1-FCD7-4195-A6D3-516CD065EAF2}"/>
     <hyperlink ref="C4" r:id="rId7" xr:uid="{41DFD0B0-9BBA-4A8B-A3BD-66F9896E3CB8}"/>
     <hyperlink ref="C5" r:id="rId8" xr:uid="{CDB1F249-484B-46AE-A525-484A9F472B8A}"/>
-    <hyperlink ref="C6" r:id="rId9" xr:uid="{7C2B7D39-0BDA-47C5-BD68-70A0F2388319}"/>
+    <hyperlink ref="C7" r:id="rId9" xr:uid="{7C2B7D39-0BDA-47C5-BD68-70A0F2388319}"/>
+    <hyperlink ref="C8" r:id="rId10" xr:uid="{79BE9E40-0586-4DCE-8052-020C8317151E}"/>
+    <hyperlink ref="C6" r:id="rId11" xr:uid="{322479B3-BFF2-4A05-BF0D-AB2C26C21215}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>